<commit_message>
Add new IMU calibration and test data files
Added multiple new data files for manual, guided, and turntable calibration and test scenarios. Renamed several existing data files for consistency. Updated data analysis scripts and added new Arduino sketches for data collection and turntable confirmation tests.
</commit_message>
<xml_diff>
--- a/IMU_CALIBATION_ALL_DATA.xlsx
+++ b/IMU_CALIBATION_ALL_DATA.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Desktop\Elu\Reaal\UT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Desktop\Elu\Reaal\UT\UT_CALIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88FB21E1-D9E1-45BE-97EC-1D95FCDBF28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD464361-7E43-45A9-90B7-6D379CC46A37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6015" yWindow="5460" windowWidth="28755" windowHeight="15435" xr2:uid="{C4B1835E-1845-4776-B4ED-FF7E979FA931}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="93">
   <si>
     <t>TEST DAY 1</t>
   </si>
@@ -309,6 +309,12 @@
   </si>
   <si>
     <t xml:space="preserve"> Success: True  Cost: 3.0194862233818176</t>
+  </si>
+  <si>
+    <t>&amp;GYRO_BIAS GX2.207271GY1.248071GZ0.380602</t>
+  </si>
+  <si>
+    <t>TEST DAY 5</t>
   </si>
 </sst>
 </file>
@@ -687,7 +693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46A04818-9C4B-4D5B-A79D-040ED7377ECE}">
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.140625" customWidth="1"/>
@@ -1189,6 +1195,26 @@
         <v>90</v>
       </c>
     </row>
+    <row r="105" spans="1:1">
+      <c r="A105" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new calibration data and update documentation
Moved calibration and reference PDFs to ALLIKAD, added new sensor and guide PDFs, introduced new calibration and accelerometer data files, updated IMU calibration spreadsheet and report, and refreshed guided/manual data and parameters for method comparison. Removed obsolete turntable parameter file and added launch configuration for gyro test.
</commit_message>
<xml_diff>
--- a/IMU_CALIBATION_ALL_DATA.xlsx
+++ b/IMU_CALIBATION_ALL_DATA.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Desktop\Elu\Reaal\UT\UT_CALIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD464361-7E43-45A9-90B7-6D379CC46A37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE43B057-AA22-4D9B-9394-22B253560B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6015" yWindow="5460" windowWidth="28755" windowHeight="15435" xr2:uid="{C4B1835E-1845-4776-B4ED-FF7E979FA931}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21000" activeTab="1" xr2:uid="{C4B1835E-1845-4776-B4ED-FF7E979FA931}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="148">
   <si>
     <t>TEST DAY 1</t>
   </si>
@@ -315,13 +316,178 @@
   </si>
   <si>
     <t>TEST DAY 5</t>
+  </si>
+  <si>
+    <t>DATA  ANALYSIS</t>
+  </si>
+  <si>
+    <t>COMMANDS:</t>
+  </si>
+  <si>
+    <t>python data_analysis_V3.py --file DATA/big_turntable_test_sample.txt --accel-file DATA/manual1.txt</t>
+  </si>
+  <si>
+    <t>Using parameters from reference run on: big_turntable_test_sample.txt</t>
+  </si>
+  <si>
+    <t>Accel: mean offset from g (calib): -0.003466</t>
+  </si>
+  <si>
+    <t>Accel: mean offset from g (raw):   0.040090</t>
+  </si>
+  <si>
+    <t>Accel: 95th%% mean abs error (calib): 0.042958</t>
+  </si>
+  <si>
+    <t>Accel: 95th%% mean abs error (raw):   0.252843</t>
+  </si>
+  <si>
+    <t>Accel: RMS fit to sphere (calib): 0.023015</t>
+  </si>
+  <si>
+    <t>Accel: RMS fit to sphere (raw):   0.136462</t>
+  </si>
+  <si>
+    <t>Params:</t>
+  </si>
+  <si>
+    <t>7.72898650e-03 -1.31745961e-01 -1.28744674e-01 9.96995134e-01 9.97720064e-01 9.90528954e-01 1.63987347e-03 -2.19314074e-03 -2.21549500e-03</t>
+  </si>
+  <si>
+    <t>python data_analysis_V3.py --file DATA/big_turntable_test_sample.txt --accel-file DATA/manual2.txt</t>
+  </si>
+  <si>
+    <t>1.73797644e-03 -1.37771053e-01 -1.48629030e-01 9.98160419e-01 9.97559960e-01 9.90269011e-01 1.45876946e-03 -3.58944324e-03 8.15213828e-04</t>
+  </si>
+  <si>
+    <t>Accel: mean offset from g (calib): -0.001355</t>
+  </si>
+  <si>
+    <t>Accel: 95th%% mean abs error (calib): 0.041541</t>
+  </si>
+  <si>
+    <t>Accel: RMS fit to sphere (calib): 0.019948</t>
+  </si>
+  <si>
+    <t>python data_analysis_V3.py --file DATA/big_turntable_test_sample.txt --accel-file DATA/MANUAL3_ACCEL.txt</t>
+  </si>
+  <si>
+    <t>1.94655176e-02 -1.38498687e-01 -1.77081956e-01 9.96840994e-01 9.97969450e-01 9.92455597e-01 3.84901151e-04 -2.47208826e-03 -1.79370363e-04</t>
+  </si>
+  <si>
+    <t>Accel: mean offset from g (calib): 0.002781</t>
+  </si>
+  <si>
+    <t>Accel: 95th%% mean abs error (calib): 0.051760</t>
+  </si>
+  <si>
+    <t>Accel: RMS fit to sphere (calib): 0.022728</t>
+  </si>
+  <si>
+    <t>MANUAL:</t>
+  </si>
+  <si>
+    <t>GUIDED:</t>
+  </si>
+  <si>
+    <t>python data_analysis_V3.py --file DATA/big_turntable_test_sample.txt --accel-file DATA/guided1.txt</t>
+  </si>
+  <si>
+    <t>Accel: mean offset from g (calib): 0.000408</t>
+  </si>
+  <si>
+    <t>Accel: 95th%% mean abs error (calib): 0.051389</t>
+  </si>
+  <si>
+    <t>Accel: RMS fit to sphere (calib): 0.025270</t>
+  </si>
+  <si>
+    <t>python data_analysis_V3.py --file DATA/big_turntable_test_sample.txt --accel-file DATA/guided2.txt</t>
+  </si>
+  <si>
+    <t>-3.13593111e-03 -1.43908572e-01 -1.66847034e-01 9.97832917e-01 9.97635081e-01 9.92246167e-01 -3.92565332e-05 -2.15197017e-03 4.87079834e-04</t>
+  </si>
+  <si>
+    <t>-3.53569221e-03 -1.30446830e-01 -1.53933907e-01 9.97342195e-01 9.97334754e-01 9.92096110e-01 7.61337394e-05 -4.16120796e-03 2.98310552e-04</t>
+  </si>
+  <si>
+    <t>Accel: mean offset from g (calib): 0.003829</t>
+  </si>
+  <si>
+    <t>Accel: 95th%% mean abs error (calib): 0.046917</t>
+  </si>
+  <si>
+    <t>Accel: RMS fit to sphere (calib): 0.023210</t>
+  </si>
+  <si>
+    <t>python data_analysis_V3.py --file DATA/big_turntable_test_sample.txt --accel-file DATA/guided3.txt</t>
+  </si>
+  <si>
+    <t>-6.17523920e-03 -1.41263564e-01 -1.78929144e-01 9.97568380e-01 9.97678031e-01 9.92155565e-01 3.61831531e-04 -2.46959521e-03 -2.98428350e-04</t>
+  </si>
+  <si>
+    <t>Accel: mean offset from g (calib): 0.002900</t>
+  </si>
+  <si>
+    <t>Accel: 95th%% mean abs error (calib): 0.055200</t>
+  </si>
+  <si>
+    <t>Accel: RMS fit to sphere (calib): 0.027670</t>
+  </si>
+  <si>
+    <t>TURNTABLE:</t>
+  </si>
+  <si>
+    <t>python data_analysis_V3.py --file DATA/big_turntable_test_sample.txt --accel-file DATA/TURNTABLE1_ACCEL.txt</t>
+  </si>
+  <si>
+    <t>python data_analysis_V3.py --file DATA/big_turntable_test_sample.txt --accel-file DATA/TURNTABLE2_ACCEL.txt</t>
+  </si>
+  <si>
+    <t>python data_analysis_V3.py --file DATA/big_turntable_test_sample.txt --accel-file DATA/TURNTABLE3_ACCEL.txt</t>
+  </si>
+  <si>
+    <t>Accel: mean offset from g (calib): -0.001743</t>
+  </si>
+  <si>
+    <t>Accel: 95th%% mean abs error (calib): 0.049929</t>
+  </si>
+  <si>
+    <t>Accel: RMS fit to sphere (calib): 0.022161</t>
+  </si>
+  <si>
+    <t>3.05352369e-02 -1.30510460e-01 -1.62633195e-01 9.97836533e-01 9.97665618e-01 9.90359965e-01 2.19241644e-03 -3.18093248e-03 2.35448411e-03</t>
+  </si>
+  <si>
+    <t>Accel: mean offset from g (calib): 0.004049</t>
+  </si>
+  <si>
+    <t>Accel: 95th%% mean abs error (calib): 0.048241</t>
+  </si>
+  <si>
+    <t>Accel: RMS fit to sphere (calib): 0.019212</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>2.59052588e-02 -1.48293908e-01 -1.72857521e-01 9.97493911e-01 9.97486188e-01 9.92835178e-01 2.55881058e-04 -2.63890016e-03 4.96229208e-04</t>
+  </si>
+  <si>
+    <t>Accel: mean offset from g (calib): -0.000923</t>
+  </si>
+  <si>
+    <t>Accel: 95th%% mean abs error (calib): 0.027933</t>
+  </si>
+  <si>
+    <t>Accel: RMS fit to sphere (calib): 0.014047</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -332,6 +498,14 @@
     <font>
       <sz val="10"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -354,11 +528,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -693,7 +868,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46A04818-9C4B-4D5B-A79D-040ED7377ECE}">
-  <dimension ref="A1:E108"/>
+  <dimension ref="A1:E126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.140625" customWidth="1"/>
@@ -1215,6 +1390,431 @@
         <v>23</v>
       </c>
     </row>
+    <row r="111" spans="1:1">
+      <c r="A111" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1">
+      <c r="A123" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126" t="s">
+        <v>95</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE5AA6E1-33C4-4A0B-BFF6-6ACD5AAFA646}">
+  <dimension ref="A1:C41"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="129.42578125" customWidth="1"/>
+    <col min="2" max="2" width="138.85546875" customWidth="1"/>
+    <col min="3" max="3" width="130" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" t="s">
+        <v>96</v>
+      </c>
+      <c r="C9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" t="s">
+        <v>118</v>
+      </c>
+      <c r="C10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>100</v>
+      </c>
+      <c r="B13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C13" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" t="s">
+        <v>120</v>
+      </c>
+      <c r="C14" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>102</v>
+      </c>
+      <c r="B15" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" t="s">
+        <v>122</v>
+      </c>
+      <c r="C19" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>96</v>
+      </c>
+      <c r="B22" t="s">
+        <v>96</v>
+      </c>
+      <c r="C22" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>107</v>
+      </c>
+      <c r="B23" t="s">
+        <v>124</v>
+      </c>
+      <c r="C23" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>98</v>
+      </c>
+      <c r="B24" t="s">
+        <v>98</v>
+      </c>
+      <c r="C24" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>108</v>
+      </c>
+      <c r="B25" t="s">
+        <v>125</v>
+      </c>
+      <c r="C25" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>100</v>
+      </c>
+      <c r="B26" t="s">
+        <v>100</v>
+      </c>
+      <c r="C26" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>109</v>
+      </c>
+      <c r="B27" t="s">
+        <v>126</v>
+      </c>
+      <c r="C27" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>102</v>
+      </c>
+      <c r="B28" t="s">
+        <v>102</v>
+      </c>
+      <c r="C28" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>111</v>
+      </c>
+      <c r="B32" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="C33" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>96</v>
+      </c>
+      <c r="B35" t="s">
+        <v>96</v>
+      </c>
+      <c r="C35" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>112</v>
+      </c>
+      <c r="B36" t="s">
+        <v>129</v>
+      </c>
+      <c r="C36" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>98</v>
+      </c>
+      <c r="B37" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>113</v>
+      </c>
+      <c r="B38" t="s">
+        <v>130</v>
+      </c>
+      <c r="C38" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>100</v>
+      </c>
+      <c r="B39" t="s">
+        <v>100</v>
+      </c>
+      <c r="C39" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>114</v>
+      </c>
+      <c r="B40" t="s">
+        <v>131</v>
+      </c>
+      <c r="C40" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>102</v>
+      </c>
+      <c r="B41" t="s">
+        <v>102</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
gyro tests and code for gyro tests
</commit_message>
<xml_diff>
--- a/IMU_CALIBATION_ALL_DATA.xlsx
+++ b/IMU_CALIBATION_ALL_DATA.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danie\Desktop\Elu\Reaal\UT\UT_CALIB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE43B057-AA22-4D9B-9394-22B253560B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA5F661-30C8-46B1-87B0-87AB5B96F97F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21000" activeTab="1" xr2:uid="{C4B1835E-1845-4776-B4ED-FF7E979FA931}"/>
+    <workbookView xWindow="4680" yWindow="4680" windowWidth="28755" windowHeight="15435" xr2:uid="{C4B1835E-1845-4776-B4ED-FF7E979FA931}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>